<commit_message>
feat: add data processing scripts, analysis reports, visualizations, and pandas reference documentation
</commit_message>
<xml_diff>
--- a/data/processed/group_table.xlsx
+++ b/data/processed/group_table.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Administrasi Bisnis</t>
+          <t>D3 - Administrasi Bisnis</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Administrasi Bisnis Otomotif</t>
+          <t>D4 - Administrasi Bisnis Otomotif</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Administrasi Negara</t>
+          <t>D4 - Administrasi Negara</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Akuntansi</t>
+          <t>D3 - Akuntansi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Akuntansi</t>
+          <t>D4 - Akuntansi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Budi Daya Ikan (Sukamara)</t>
+          <t>D3 - Budi Daya Ikan (Sukamara)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Teknologi Budidaya Perikanan</t>
+          <t>D3 - Teknik Sipil</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -586,7 +586,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Teknologi Budidaya Perikanan (Kapuas Hulu)</t>
+          <t>D3 - Teknologi Budidaya Perikanan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10">
@@ -606,7 +606,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Teknologi Penangkapan Ikan</t>
+          <t>D3 - Teknologi Budidaya Perikanan (Kapuas Hulu)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -626,7 +626,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Teknologi Pengolahan Hasil Perikanan</t>
+          <t>D3 - Teknologi Penangkapan Ikan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -635,18 +635,18 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Teknik Arsitektur</t>
+          <t>Ilmu Kelautan dan Perikanan</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Arsitektur</t>
+          <t>D3 - Teknologi Pengolahan Hasil Perikanan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -666,16 +666,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Arsitektur Bangunan Gedung</t>
+          <t>D3 - Arsitektur</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14">
@@ -686,7 +686,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Desain Kawasan Binaan</t>
+          <t>D4 - Arsitektur Bangunan Gedung</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -695,27 +695,27 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Teknik Elektro</t>
+          <t>Teknik Arsitektur</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Teknik Elektronika</t>
+          <t>D4 - Desain Kawasan Binaan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -726,7 +726,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Teknik Informatika</t>
+          <t>D3 - Teknik Elektronika</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
@@ -746,7 +746,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Teknik Listrik</t>
+          <t>D3 - Teknik Informatika</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18">
@@ -766,36 +766,36 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Teknologi Rekayasa Sistem Elektronika</t>
+          <t>D3 - Teknik Listrik</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Teknik Mesin</t>
+          <t>Teknik Elektro</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Operator dan Peralatan Alat Berat</t>
+          <t>D4 - Teknologi Rekayasa Sistem Elektronika</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20">
@@ -806,16 +806,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pemeliharaan Kendaraan Ringan</t>
+          <t>D1 - Operator dan Peralatan Alat Berat</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21">
@@ -826,16 +826,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Teknik Mesin</t>
+          <t>D2 - Pemeliharaan Kendaraan Ringan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -846,16 +846,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Teknik Mesin</t>
+          <t>D3 - Teknik Mesin</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23">
@@ -866,7 +866,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Teknologi Mesin (Sanggau)</t>
+          <t>D3 - Teknologi Mesin (Sanggau)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -881,12 +881,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Teknik Sipil dan Perencanaan</t>
+          <t>Teknik Mesin</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Perencanaan Perumahan Dan Pemukiman</t>
+          <t>D4 - Teknik Mesin</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25">
@@ -906,7 +906,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Teknik Sipil</t>
+          <t>D3 - Teknik Sipil</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -915,18 +915,18 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Teknologi Pertanian</t>
+          <t>Teknik Sipil dan Perencanaan</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Budidaya Tanaman Perkebunan</t>
+          <t>D4 - Perencanaan Perumahan Dan Pemukiman</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -935,7 +935,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>24</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27">
@@ -946,16 +946,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Manajemen Perkebunan</t>
+          <t>D3 - Teknologi Pengolahan Hasil Perkebunan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
@@ -966,7 +966,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Pengolahan Hasil Perkebunan Terpadu</t>
+          <t>D4 - Budidaya Tanaman Perkebunan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29">
@@ -986,16 +986,36 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Teknologi Pengolahan Hasil Perkebunan</t>
+          <t>D4 - Manajemen Perkebunan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>7</v>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Teknologi Pertanian</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>D4 - Pengolahan Hasil Perkebunan Terpadu</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add viz_utils.py and supporting visualization scripts to generate map-based and statistical reports for alumni tracer data.
</commit_message>
<xml_diff>
--- a/data/processed/group_table.xlsx
+++ b/data/processed/group_table.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -566,7 +566,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>D3 - Teknik Sipil</t>
+          <t>D3 - Teknologi Budidaya Perikanan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
@@ -586,7 +586,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>D3 - Teknologi Budidaya Perikanan</t>
+          <t>D3 - Teknologi Budidaya Perikanan (Kapuas Hulu)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -606,7 +606,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>D3 - Teknologi Budidaya Perikanan (Kapuas Hulu)</t>
+          <t>D3 - Teknologi Penangkapan Ikan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
@@ -626,7 +626,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>D3 - Teknologi Penangkapan Ikan</t>
+          <t>D3 - Teknologi Pengolahan Hasil Perikanan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -635,18 +635,18 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ilmu Kelautan dan Perikanan</t>
+          <t>Teknik Arsitektur</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>D3 - Teknologi Pengolahan Hasil Perikanan</t>
+          <t>D3 - Arsitektur</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13">
@@ -666,16 +666,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>D3 - Arsitektur</t>
+          <t>D4 - Arsitektur Bangunan Gedung</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
@@ -686,7 +686,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>D4 - Arsitektur Bangunan Gedung</t>
+          <t>D4 - Desain Kawasan Binaan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -695,27 +695,27 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Teknik Arsitektur</t>
+          <t>Teknik Elektro</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>D4 - Desain Kawasan Binaan</t>
+          <t>D3 - Teknik Elektronika</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -726,7 +726,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>D3 - Teknik Elektronika</t>
+          <t>D3 - Teknik Informatika</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17">
@@ -746,7 +746,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>D3 - Teknik Informatika</t>
+          <t>D3 - Teknik Listrik</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18">
@@ -766,36 +766,36 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>D3 - Teknik Listrik</t>
+          <t>D4 - Teknologi Rekayasa Sistem Elektronika</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Teknik Elektro</t>
+          <t>Teknik Mesin</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>D4 - Teknologi Rekayasa Sistem Elektronika</t>
+          <t>D1 - Operator dan Peralatan Alat Berat</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -806,16 +806,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>D1 - Operator dan Peralatan Alat Berat</t>
+          <t>D2 - Pemeliharaan Kendaraan Ringan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -826,16 +826,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>D2 - Pemeliharaan Kendaraan Ringan</t>
+          <t>D3 - Teknik Mesin</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22">
@@ -846,7 +846,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>D3 - Teknik Mesin</t>
+          <t>D3 - Teknologi Mesin (Sanggau)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -866,36 +866,36 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>D3 - Teknologi Mesin (Sanggau)</t>
+          <t>D4 - Teknik Mesin</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Teknik Mesin</t>
+          <t>Teknik Sipil dan Perencanaan</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>D4 - Teknik Mesin</t>
+          <t>D3 - Teknik Sipil</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25">
@@ -906,36 +906,36 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>D3 - Teknik Sipil</t>
+          <t>D4 - Perencanaan Perumahan Dan Pemukiman</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>14</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Teknik Sipil dan Perencanaan</t>
+          <t>Teknologi Pertanian</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>D4 - Perencanaan Perumahan Dan Pemukiman</t>
+          <t>D3 - Teknologi Pengolahan Hasil Perkebunan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>41</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27">
@@ -946,16 +946,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>D3 - Teknologi Pengolahan Hasil Perkebunan</t>
+          <t>D4 - Budidaya Tanaman Perkebunan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28">
@@ -966,7 +966,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>D4 - Budidaya Tanaman Perkebunan</t>
+          <t>D4 - Manajemen Perkebunan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>24</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29">
@@ -986,7 +986,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>D4 - Manajemen Perkebunan</t>
+          <t>D4 - Pengolahan Hasil Perkebunan Terpadu</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -995,26 +995,6 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Teknologi Pertanian</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>D4 - Pengolahan Hasil Perkebunan Terpadu</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>D4</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
         <v>32</v>
       </c>
     </row>

</xml_diff>